<commit_message>
add new filter tests
</commit_message>
<xml_diff>
--- a/selenium-tests/test-cases.xlsx
+++ b/selenium-tests/test-cases.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="221">
   <si>
     <t>ID</t>
   </si>
@@ -3271,7 +3271,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" ht="128.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" ht="128.25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>195</v>
       </c>
@@ -3294,9 +3294,14 @@
       <c r="H5" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" ht="128.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="J5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" ht="128.25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>199</v>
       </c>
@@ -3321,7 +3326,12 @@
       <c r="H6" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="I6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="J6" t="s">
+        <v>120</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
add new register test
</commit_message>
<xml_diff>
--- a/selenium-tests/test-cases.xlsx
+++ b/selenium-tests/test-cases.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00E671D-820B-4CFB-858C-0A95B39A69A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="6" name="Login" state="visible" r:id="rId4"/>
-    <sheet sheetId="7" name="Register" state="visible" r:id="rId5"/>
-    <sheet sheetId="5" name="Cart" state="visible" r:id="rId6"/>
-    <sheet sheetId="3" name="Checkout" state="visible" r:id="rId7"/>
-    <sheet sheetId="8" name="Filter" state="visible" r:id="rId8"/>
-    <sheet sheetId="10" name="Order" state="visible" r:id="rId9"/>
-    <sheet sheetId="12" name="IntegratedTests" state="visible" r:id="rId10"/>
+    <sheet name="Login" sheetId="6" r:id="rId1"/>
+    <sheet name="Register" sheetId="7" r:id="rId2"/>
+    <sheet name="Cart" sheetId="5" r:id="rId3"/>
+    <sheet name="Checkout" sheetId="3" r:id="rId4"/>
+    <sheet name="Filter" sheetId="8" r:id="rId5"/>
+    <sheet name="Order" sheetId="10" r:id="rId6"/>
+    <sheet name="IntegratedTests" sheetId="12" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="167">
   <si>
     <t>ID</t>
   </si>
@@ -61,7 +62,7 @@
     <t>Đã có tài khoản</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng nhập (localhost:4200/login)
 3.	Xác nhận trang đăng nhập hiển thị thành công
 4.	Nhập thông tin đăng nhập
@@ -88,7 +89,7 @@
     <t>Đăng nhập với email sai</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng nhập (localhost:4200/login)
 3.	Xác nhận trang đăng nhập hiển thị thành công
 4.	Nhập thông tin đăng nhập với email không hợp lệ
@@ -107,7 +108,7 @@
     <t>Đăng nhập với email bỏ trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng nhập (localhost:4200/login)
 3.	Xác nhận trang đăng nhập hiển thị thành công
 4.	Nhập thông tin đăng nhập với email bỏ trống
@@ -123,7 +124,7 @@
     <t>Đăng nhập với mật khẩu bỏ trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng nhập (localhost:4200/login)
 3.	Xác nhận trang đăng nhập hiển thị thành công
 4.	Nhập thông tin đăng nhập với mật khẩu bỏ trống
@@ -139,7 +140,7 @@
     <t>Đăng nhập với email định dạng không hợp lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng nhập (localhost:4200/login)
 3.	Xác nhận trang đăng nhập hiển thị thành công
 4.	Nhập thông tin đăng nhập với email "nguyenquocthang909@gmail."
@@ -158,7 +159,7 @@
     <t>Đăng nhập với mật khẩu định dạng không hợp lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng nhập (localhost:4200/login)
 3.	Xác nhận trang đăng nhập hiển thị thành công
 4.	Nhập thông tin đăng nhập với mật khẩu "12345"
@@ -177,7 +178,7 @@
     <t>Đăng ký vói thông tin hợp lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng ký (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký
@@ -197,7 +198,7 @@
     <t>Đăng ký với mật khẩu không khớp</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng Nhập (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký với mật khẩu và xác nhận mật khẩu không khớp
@@ -213,7 +214,7 @@
     <t>Đăng ký với email bỏ trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng Nhập (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký với email bỏ trống
@@ -226,7 +227,7 @@
     <t>Đăng ký với mật khẩu bỏ trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng Nhập (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký với mật khẩu bỏ trống
@@ -239,7 +240,7 @@
     <t>Đăng ký với email định dạng không hợp lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng Nhập (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký với email "nguyenquocthang909@gmail."
@@ -252,7 +253,7 @@
     <t>Đăng ký với mật khẩu định dạng không hợp lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng Nhập (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký với mật khẩu và xác nhận mật khẩu "12345"
@@ -265,7 +266,7 @@
     <t>Đăng ký với thông tin đăng ký của một tài khoản đã có tồn tại trong CSDL</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang đăng Nhập (localhost:4200/register)
 3.	Xác nhận trang đăng ký hiển thị thành công
 4.	Nhập thông tin đăng ký đã tồn tại
@@ -284,11 +285,11 @@
     <t>Thêm vào giỏ hàng thành công</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
+    <t>Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
 Sản phẩm có tồn kho lớn hơn 0</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang hiển thị thành công
 4.	Bấm nút đăng nhập
@@ -312,11 +313,11 @@
     <t>Sản phẩm có trong giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
+    <t>Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
 Có ít nhất 1 sản phẩm trong giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm A
@@ -337,11 +338,11 @@
     <t>Tăng SL sản phẩm từ giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
+    <t>Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
 Có ít nhất 1 sản phẩm với số lượng lớn hơn 0 trong giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang hiển thị thành công
 4.	Xác nhận trang bán hoa hiển thị thành công
@@ -367,11 +368,11 @@
     <t>Giảm SL sản phẩm từ giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
+    <t>Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
 Có ít nhất 1 sản phẩm với số lượng lớn hơn 1 trong giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm A
@@ -396,7 +397,7 @@
     <t>Xoá sản phẩm từ giỏ hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm A
@@ -433,7 +434,7 @@
     <t>Thanh toán thành công</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -481,12 +482,12 @@
     <t>Thanh toán với voucher hết hạn</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
+    <t>Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa
 Có ít nhất 1 sản phẩm trong giỏ hàng
 Có ít nhất 1 voucher</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -519,7 +520,7 @@
     <t>Thanh toán với thông tin thanh toán trường nhập họ để trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -545,7 +546,7 @@
     <t>Thanh toán với thông tin thanh toán trường nhập tên để trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -571,7 +572,7 @@
     <t>Thanh toán với thông tin thanh toán trường nhập email để trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -600,7 +601,7 @@
     <t>Thanh toán với thông tin thanh toán trường nhập SĐT để trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -632,7 +633,7 @@
     <t>Thanh toán với thông tin thanh toán trường nhập ghi chú để trống</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Truy cập trang chi tiết sản phẩm ngẫu nhiên
@@ -664,7 +665,7 @@
     <t>Đã có tài khoản và đang trong phiên đăng nhập với trang bán hoa</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Xác nhận thanh tìm kiếm hiển thị thành công
@@ -685,7 +686,7 @@
     <t>Tìm kiếm sản phẩm với từ khoá không tồn tại trong các sản phẩm</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Xác nhận thanh tìm kiếm hiển thị thành công
@@ -706,7 +707,7 @@
     <t>Tìm kiếm và lọc sản phẩm theo giá</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Kéo thanh lọc giá đến giá trị định sẵn
@@ -725,7 +726,7 @@
     <t>Tìm kiếm và lọc sản phẩm theo giá với từ khoá</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Kéo thanh lọc giá đến giá trị định sẵn
@@ -741,7 +742,7 @@
     <t>Xem chi tiết đơn hàng được làm nổi bật</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Xác nhận hình cá nhân hiển thị thành công
@@ -762,7 +763,7 @@
     <t>Huỷ đơn hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Xác nhận hình cá nhân hiển thị thành công
@@ -788,7 +789,7 @@
     <t>Huỷ đơn hàng không có lý do</t>
   </si>
   <si>
-    <t xml:space="preserve">1.	Mở trình duyệt tùy chọn
+    <t>1.	Mở trình duyệt tùy chọn
 2.	Truy cập trang bán hoa (localhost:4200)
 3.	Xác nhận trang bán hoa hiển thị thành công
 4.	Xác nhận hình cá nhân hiển thị thành công
@@ -822,44 +823,44 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="0"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Arial"/>
-    </font>
-    <font>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -974,7 +975,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1006,38 +1007,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1059,6 +1030,42 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1392,225 +1399,760 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.75" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.25" style="2" customWidth="1"/>
-    <col min="4" max="4" width="31.75" style="2" customWidth="1"/>
-    <col min="5" max="5" width="33.375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="23.875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.5" style="2" customWidth="1"/>
-    <col min="9" max="9" width="6.5" style="2" customWidth="1"/>
+    <col min="1" max="1" width="17.875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.75" style="3" customWidth="1"/>
+    <col min="5" max="5" width="29.125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="39.125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="35.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="19" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="21"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-    </row>
-    <row r="3" ht="243" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>151</v>
+      <c r="G2" s="20"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="100.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>135</v>
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="E3" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="8" t="s">
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>154</v>
+        <v>16</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" ht="384.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>155</v>
+        <v>16</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>135</v>
+        <v>19</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="E4" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F6" s="8"/>
+      <c r="G6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="356.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="E5" s="25" t="s">
+      <c r="G7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>162</v>
-      </c>
+      <c r="F8" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="114" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="6"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="8"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="8"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="6"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="8"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="6"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D14" s="6"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="8"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D15" s="6"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D16" s="6"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.875" customWidth="1"/>
-    <col min="2" max="2" width="36.625" style="27" customWidth="1"/>
-    <col min="3" max="8" width="17.875" customWidth="1"/>
+    <col min="1" max="1" width="7.75" style="9" customWidth="1"/>
+    <col min="2" max="2" width="29.875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14" style="9" customWidth="1"/>
+    <col min="4" max="4" width="40.75" style="9" customWidth="1"/>
+    <col min="5" max="6" width="29.75" style="9" customWidth="1"/>
+    <col min="7" max="7" width="24.875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="24.875" style="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8.875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.75" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27" style="2" customWidth="1"/>
+    <col min="4" max="4" width="40.75" style="2" customWidth="1"/>
+    <col min="5" max="5" width="32.875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17" style="2" customWidth="1"/>
+    <col min="7" max="8" width="26.5" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.5" style="2" customWidth="1"/>
+    <col min="10" max="10" width="17.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="H1" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="I1" s="23" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="29.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+    </row>
+    <row r="3" spans="1:9" ht="285.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="3" ht="28.5" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="4" ht="28.5" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="27" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" ht="28.5" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="27" t="s">
-        <v>166</v>
-      </c>
+      <c r="B3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="242.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="270.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="270.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="256.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="185.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C8" s="10"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8"/>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.25" style="1" customWidth="1"/>
     <col min="2" max="2" width="19.75" style="2" customWidth="1"/>
@@ -1628,43 +2170,43 @@
     <col min="15" max="15" width="17.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="5" t="s">
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="19" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="20"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="21"/>
+    <row r="2" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="27"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="29"/>
       <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
@@ -1686,11 +2228,11 @@
       <c r="K2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="4"/>
-    </row>
-    <row r="3" ht="357" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="19"/>
+    </row>
+    <row r="3" spans="1:14" ht="357" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>93</v>
       </c>
@@ -1734,7 +2276,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" ht="356.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="356.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>103</v>
       </c>
@@ -1778,7 +2320,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>109</v>
       </c>
@@ -1820,7 +2362,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>113</v>
       </c>
@@ -1862,7 +2404,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>117</v>
       </c>
@@ -1875,7 +2417,7 @@
       <c r="D7" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="12" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1906,7 +2448,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>120</v>
       </c>
@@ -1919,7 +2461,7 @@
       <c r="D8" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="12" t="s">
         <v>14</v>
       </c>
       <c r="F8" s="8" t="s">
@@ -1950,7 +2492,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>122</v>
       </c>
@@ -1992,7 +2534,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>126</v>
       </c>
@@ -2034,7 +2576,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" ht="285" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="285" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>128</v>
       </c>
@@ -2078,756 +2620,23 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="L1:L2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
     <mergeCell ref="E1:K1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="L1:L2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="8.875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.75" style="2" customWidth="1"/>
-    <col min="3" max="3" width="27" style="2" customWidth="1"/>
-    <col min="4" max="4" width="40.75" style="2" customWidth="1"/>
-    <col min="5" max="5" width="32.875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="17" style="2" customWidth="1"/>
-    <col min="7" max="8" width="26.5" style="2" customWidth="1"/>
-    <col min="9" max="9" width="6.5" style="2" customWidth="1"/>
-    <col min="10" max="10" width="17.875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="15"/>
-      <c r="G1" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-    </row>
-    <row r="3" ht="285.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" ht="242.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="270.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" ht="270.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" ht="256.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" ht="185.25" customHeight="1" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="10"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="8"/>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="17.875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="35.5" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.875" style="1" customWidth="1"/>
-    <col min="4" max="6" width="44.75" style="3" customWidth="1"/>
-    <col min="7" max="7" width="39.125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="35.625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="17.875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-    </row>
-    <row r="3" ht="100.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" ht="71.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="71.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" ht="71.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" ht="85.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" ht="71.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" ht="114" customHeight="1" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D9" s="6"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="8"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" ht="85.5" customHeight="1" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="8"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" ht="99.75" customHeight="1" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="8"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" ht="85.5" customHeight="1" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="8"/>
-    </row>
-    <row r="13" ht="85.5" customHeight="1" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D13" s="6"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" ht="99.75" customHeight="1" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D14" s="6"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="8"/>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" ht="99.75" customHeight="1" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D15" s="6"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" ht="85.5" customHeight="1" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D16" s="6"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="8"/>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="7.75" style="9" customWidth="1"/>
-    <col min="2" max="2" width="29.875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14" style="9" customWidth="1"/>
-    <col min="4" max="4" width="40.75" style="9" customWidth="1"/>
-    <col min="5" max="6" width="29.75" style="9" customWidth="1"/>
-    <col min="7" max="7" width="25.375" style="9" customWidth="1"/>
-    <col min="8" max="8" width="17.875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-    </row>
-    <row r="3" ht="99.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" ht="85.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-    </row>
-    <row r="5" ht="85.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-    </row>
-    <row r="6" ht="99.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-    </row>
-    <row r="7" ht="99.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-    </row>
-    <row r="8" ht="85.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-    </row>
-    <row r="9" ht="14.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5" style="2" customWidth="1"/>
     <col min="2" max="3" width="36.625" style="2" customWidth="1"/>
@@ -2839,53 +2648,53 @@
     <col min="10" max="10" width="6.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="13" t="s">
+      <c r="F1" s="25"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="23" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="23" t="s">
+    <row r="2" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="23" t="s">
+      <c r="G2" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-    </row>
-    <row r="3" ht="129" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+    </row>
+    <row r="3" spans="1:10" ht="129" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>133</v>
       </c>
@@ -2917,7 +2726,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" ht="114" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="114" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>139</v>
       </c>
@@ -2949,11 +2758,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="128.25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="14" t="s">
         <v>145</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2978,11 +2787,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" ht="128.25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="14" t="s">
         <v>149</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3012,15 +2821,230 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.75" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.25" style="2" customWidth="1"/>
+    <col min="4" max="4" width="31.75" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33.375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="23.875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.5" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.5" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="29"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+    </row>
+    <row r="3" spans="1:9" ht="243" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="384.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="356.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.875" customWidth="1"/>
+    <col min="2" max="2" width="36.625" style="17" customWidth="1"/>
+    <col min="3" max="8" width="17.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="17" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="17" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>